<commit_message>
chore: update TestProject excel config files
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -1,35 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E906D24-9650-440B-98FF-54828A9FCE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0048B3F-23D4-423D-83A0-B1C15A3C963E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2630" yWindow="1020" windowWidth="34360" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10470" yWindow="1450" windowWidth="27140" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PIParameters" sheetId="1" r:id="rId1"/>
-    <sheet name="PIOutputMappings" sheetId="2" r:id="rId2"/>
-    <sheet name="PIConfiguration" sheetId="3" r:id="rId3"/>
+    <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
+    <sheet name="PIParameters" sheetId="2" r:id="rId2"/>
+    <sheet name="PIOutputMappings" sheetId="3" r:id="rId3"/>
     <sheet name="AlgorithmOptions" sheetId="4" r:id="rId4"/>
     <sheet name="CIOptions" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
   <si>
     <t>PITaskName</t>
   </si>
   <si>
-    <t>Scenario</t>
+    <t>Algorithm</t>
+  </si>
+  <si>
+    <t>CIMethod</t>
+  </si>
+  <si>
+    <t>PrintEvaluationFeedback</t>
+  </si>
+  <si>
+    <t>AutoEstimateCI</t>
+  </si>
+  <si>
+    <t>SimulationRunOptions</t>
+  </si>
+  <si>
+    <t>ObjectiveFunctionOptions</t>
+  </si>
+  <si>
+    <t>AciclovirSimple</t>
+  </si>
+  <si>
+    <t>BOBYQA</t>
+  </si>
+  <si>
+    <t>hessian</t>
+  </si>
+  <si>
+    <t>Scenarios</t>
   </si>
   <si>
     <t>Container Path</t>
@@ -56,9 +83,6 @@
     <t>Group</t>
   </si>
   <si>
-    <t>AciclovirLinear</t>
-  </si>
-  <si>
     <t>PITestScenario</t>
   </si>
   <si>
@@ -71,12 +95,27 @@
     <t>Log Units</t>
   </si>
   <si>
-    <t>AciclovirLog</t>
+    <t>AciclovirMultiScenario</t>
+  </si>
+  <si>
+    <t>PIScenario_250mg</t>
+  </si>
+  <si>
+    <t>PIScenario_500mg</t>
+  </si>
+  <si>
+    <t>Neighborhoods|Kidney_pls_Kidney_ur|Aciclovir|Renal Clearances-TS</t>
+  </si>
+  <si>
+    <t>TSspec</t>
   </si>
   <si>
     <t>ObservedDataSheet</t>
   </si>
   <si>
+    <t>DataSet</t>
+  </si>
+  <si>
     <t>Scaling</t>
   </si>
   <si>
@@ -92,37 +131,16 @@
     <t>Laskin 1982.Group A</t>
   </si>
   <si>
+    <t>Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_2.5 mg/kg_iv_</t>
+  </si>
+  <si>
+    <t>log</t>
+  </si>
+  <si>
     <t>lin</t>
   </si>
   <si>
-    <t>log</t>
-  </si>
-  <si>
-    <t>Algorithm</t>
-  </si>
-  <si>
-    <t>CIMethod</t>
-  </si>
-  <si>
-    <t>PrintEvaluationFeedback</t>
-  </si>
-  <si>
-    <t>AutoEstimateCI</t>
-  </si>
-  <si>
-    <t>SimulationRunOptions</t>
-  </si>
-  <si>
-    <t>ObjectiveFunctionOptions</t>
-  </si>
-  <si>
-    <t>BOBYQA</t>
-  </si>
-  <si>
-    <t>hessian</t>
-  </si>
-  <si>
-    <t>TRUE</t>
+    <t>Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_5.0 mg/kg_iv_</t>
   </si>
   <si>
     <t>OptionName</t>
@@ -138,21 +156,23 @@
   </si>
   <si>
     <t>confLevel</t>
-  </si>
-  <si>
-    <t>Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_2.5 mg/kg_iv_</t>
-  </si>
-  <si>
-    <t>DataSet</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -181,13 +201,15 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -200,9 +222,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -240,7 +262,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -312,7 +334,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -344,16 +366,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -475,338 +501,383 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.9140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.75" bestFit="1" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="1">
-        <v>-0.1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2">
-        <v>-10</v>
-      </c>
-      <c r="H2">
-        <v>10</v>
-      </c>
-      <c r="I2">
+      <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3">
-        <v>-10</v>
-      </c>
-      <c r="H3">
-        <v>10</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
+      <c r="E2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:J1 E3:F3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.9140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.9140625" customWidth="1"/>
-    <col min="4" max="4" width="23.33203125" customWidth="1"/>
-    <col min="5" max="6" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.58203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.26953125" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2">
+        <v>-0.1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2">
+        <v>-10</v>
+      </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+      <c r="I2">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="J2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3">
+        <v>-0.1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3">
+        <v>-10</v>
+      </c>
+      <c r="H3">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="E4">
+        <v>-0.1</v>
+      </c>
+      <c r="F4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G4">
+        <v>-10</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>23</v>
       </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>0.5</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>0.5</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Only for observed data" prompt="This cell is only required for data of type 'observed', leave blank otherwise" sqref="D2:D3" xr:uid="{6B9A838E-5CC1-4104-9014-3891C5629AB5}"/>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="E1:H3 A1:C3" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="82.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="D1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" t="b">
-        <v>0</v>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G1 A3:D3 A2:D2 F2:G2 F3:G3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C1" t="s">
-        <v>34</v>
+      <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C2">
-        <v>1000</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -814,34 +885,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C1 A2:B3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C1" t="s">
-        <v>34</v>
+      <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C2">
         <v>0.95</v>
@@ -849,8 +917,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C1 A2:B2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: apply xOffset/yOffset/xFactor/yFactor to PIOutputMapping
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0048B3F-23D4-423D-83A0-B1C15A3C963E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E257BB-0E2B-4F4F-89BE-0CA5AC014FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10470" yWindow="1450" windowWidth="27140" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2190" yWindow="870" windowWidth="27140" windowHeight="19040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="46">
   <si>
     <t>PITaskName</t>
   </si>
@@ -156,6 +156,12 @@
   </si>
   <si>
     <t>confLevel</t>
+  </si>
+  <si>
+    <t>xFactor</t>
+  </si>
+  <si>
+    <t>yFactor</t>
   </si>
 </sst>
 </file>
@@ -754,7 +760,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
@@ -763,7 +769,7 @@
     <col min="4" max="4" width="82.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -786,10 +792,16 @@
         <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -806,7 +818,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -823,7 +835,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
fix: expand objective function options
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E257BB-0E2B-4F4F-89BE-0CA5AC014FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4204C60-09C9-4CA3-9F9E-1AE47E595EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2190" yWindow="870" windowWidth="27140" windowHeight="19040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2800" yWindow="960" windowWidth="27140" windowHeight="19040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="51">
   <si>
     <t>PITaskName</t>
   </si>
@@ -44,9 +44,6 @@
     <t>SimulationRunOptions</t>
   </si>
   <si>
-    <t>ObjectiveFunctionOptions</t>
-  </si>
-  <si>
     <t>AciclovirSimple</t>
   </si>
   <si>
@@ -162,6 +159,24 @@
   </si>
   <si>
     <t>yFactor</t>
+  </si>
+  <si>
+    <t>ObjectiveFunctionType</t>
+  </si>
+  <si>
+    <t>ResidualWeightingMethod</t>
+  </si>
+  <si>
+    <t>RobustMethod</t>
+  </si>
+  <si>
+    <t>ScaleVar</t>
+  </si>
+  <si>
+    <t>LinScaleCV</t>
+  </si>
+  <si>
+    <t>LogScaleSD</t>
   </si>
 </sst>
 </file>
@@ -514,10 +529,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,18 +552,33 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -577,51 +607,51 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>20</v>
-      </c>
-      <c r="D2" t="s">
-        <v>21</v>
       </c>
       <c r="E2">
         <v>-0.1</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G2">
         <v>-10</v>
@@ -638,22 +668,22 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
       <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
         <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
       </c>
       <c r="E3">
         <v>-0.1</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G3">
         <v>-10</v>
@@ -670,22 +700,22 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
         <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
       </c>
       <c r="E4">
         <v>-0.1</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4">
         <v>-10</v>
@@ -702,16 +732,16 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
       <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
         <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -728,16 +758,16 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -774,82 +804,82 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" t="s">
-        <v>35</v>
-      </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
       <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -867,18 +897,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -886,10 +916,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -910,18 +940,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2">
         <v>0.95</v>

</xml_diff>

<commit_message>
fix: add OutputPath column to PIOutputMappings
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -1,185 +1,198 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\pi-workflow\inst\extdata\examples\TestProject\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F231B5A2-57F5-42D0-9067-256CA473510A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="2080" yWindow="960" windowWidth="27640" windowHeight="19270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PIConfiguration" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PIParameters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PIOutputMappings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlgorithmOptions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CIOptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
+    <sheet name="PIParameters" sheetId="2" r:id="rId2"/>
+    <sheet name="PIOutputMappings" sheetId="3" r:id="rId3"/>
+    <sheet name="AlgorithmOptions" sheetId="4" r:id="rId4"/>
+    <sheet name="CIOptions" sheetId="5" r:id="rId5"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
-  <si>
-    <t xml:space="preserve">PITaskName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Algorithm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIMethod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrintEvaluationFeedback</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AutoEstimateCI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">numberOfCores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">checkForNegativeValues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ObjectiveFunctionType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ResidualWeightingMethod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RobustMethod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ScaleVar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinScaleCV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LogScaleSD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AciclovirSimple</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOBYQA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hessian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scenarios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Container Path</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameter Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MinValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MaxValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">StartValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PITestScenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aciclovir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lipophilicity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Log Units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AciclovirMultiScenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIScenario_250mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIScenario_500mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neighborhoods|Kidney_pls_Kidney_ur|Aciclovir|Renal Clearances-TS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TSspec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ObservedDataSheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DataSet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scaling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yOffset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xFactor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yFactor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laskin 1982.Group A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_2.5 mg/kg_iv_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">log</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_5.0 mg/kg_iv_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OptionName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OptionValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">maxeval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ftol_rel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">confLevel</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="54">
+  <si>
+    <t>PITaskName</t>
+  </si>
+  <si>
+    <t>Algorithm</t>
+  </si>
+  <si>
+    <t>CIMethod</t>
+  </si>
+  <si>
+    <t>PrintEvaluationFeedback</t>
+  </si>
+  <si>
+    <t>AutoEstimateCI</t>
+  </si>
+  <si>
+    <t>numberOfCores</t>
+  </si>
+  <si>
+    <t>checkForNegativeValues</t>
+  </si>
+  <si>
+    <t>ObjectiveFunctionType</t>
+  </si>
+  <si>
+    <t>ResidualWeightingMethod</t>
+  </si>
+  <si>
+    <t>RobustMethod</t>
+  </si>
+  <si>
+    <t>ScaleVar</t>
+  </si>
+  <si>
+    <t>LinScaleCV</t>
+  </si>
+  <si>
+    <t>LogScaleSD</t>
+  </si>
+  <si>
+    <t>AciclovirSimple</t>
+  </si>
+  <si>
+    <t>BOBYQA</t>
+  </si>
+  <si>
+    <t>hessian</t>
+  </si>
+  <si>
+    <t>Scenarios</t>
+  </si>
+  <si>
+    <t>Container Path</t>
+  </si>
+  <si>
+    <t>Parameter Name</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>MinValue</t>
+  </si>
+  <si>
+    <t>MaxValue</t>
+  </si>
+  <si>
+    <t>StartValue</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>PITestScenario</t>
+  </si>
+  <si>
+    <t>Aciclovir</t>
+  </si>
+  <si>
+    <t>Lipophilicity</t>
+  </si>
+  <si>
+    <t>Log Units</t>
+  </si>
+  <si>
+    <t>AciclovirMultiScenario</t>
+  </si>
+  <si>
+    <t>PIScenario_250mg</t>
+  </si>
+  <si>
+    <t>PIScenario_500mg</t>
+  </si>
+  <si>
+    <t>Neighborhoods|Kidney_pls_Kidney_ur|Aciclovir|Renal Clearances-TS</t>
+  </si>
+  <si>
+    <t>TSspec</t>
+  </si>
+  <si>
+    <t>ObservedDataSheet</t>
+  </si>
+  <si>
+    <t>DataSet</t>
+  </si>
+  <si>
+    <t>Scaling</t>
+  </si>
+  <si>
+    <t>xOffset</t>
+  </si>
+  <si>
+    <t>yOffset</t>
+  </si>
+  <si>
+    <t>xFactor</t>
+  </si>
+  <si>
+    <t>yFactor</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Laskin 1982.Group A</t>
+  </si>
+  <si>
+    <t>Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_2.5 mg/kg_iv_</t>
+  </si>
+  <si>
+    <t>lin</t>
+  </si>
+  <si>
+    <t>log</t>
+  </si>
+  <si>
+    <t>Laskin 1982.Group A_Aciclovir_1_Human_MALE_PeripheralVenousBlood_Plasma_5.0 mg/kg_iv_</t>
+  </si>
+  <si>
+    <t>OptionName</t>
+  </si>
+  <si>
+    <t>OptionValue</t>
+  </si>
+  <si>
+    <t>maxeval</t>
+  </si>
+  <si>
+    <t>ftol_rel</t>
+  </si>
+  <si>
+    <t>confLevel</t>
+  </si>
+  <si>
+    <t>OutputPath</t>
+  </si>
+  <si>
+    <t>Organism|PeripheralVenousBlood|Aciclovir|Plasma (Peripheral Venous Blood)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -215,6 +228,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -496,11 +518,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -541,7 +563,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -557,27 +579,19 @@
       <c r="E2" t="b">
         <v>0</v>
       </c>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -609,7 +623,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -622,26 +636,26 @@
       <c r="D2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>-0.1</v>
       </c>
       <c r="F2" t="s">
         <v>28</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>-10</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2">
         <v>10</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -654,26 +668,26 @@
       <c r="D3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>-0.1</v>
       </c>
       <c r="F3" t="s">
         <v>28</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>-10</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3">
         <v>10</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3">
         <v>1</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3">
         <v>1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -686,26 +700,26 @@
       <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>-0.1</v>
       </c>
       <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>-10</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4">
         <v>10</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4">
         <v>1</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4">
         <v>1</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -718,22 +732,20 @@
       <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5">
         <v>10</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5">
         <v>0.5</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5">
         <v>2</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -746,33 +758,35 @@
       <c r="D6" t="s">
         <v>33</v>
       </c>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6">
         <v>10</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6">
         <v>0.5</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -780,31 +794,34 @@
         <v>16</v>
       </c>
       <c r="C1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>37</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>38</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>39</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>40</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -812,21 +829,19 @@
         <v>25</v>
       </c>
       <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>44</v>
       </c>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-      <c r="J2"/>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -834,21 +849,19 @@
         <v>30</v>
       </c>
       <c r="C3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" t="s">
         <v>42</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>43</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>45</v>
       </c>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
-      <c r="J3"/>
-    </row>
-    <row r="4">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -856,32 +869,30 @@
         <v>31</v>
       </c>
       <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
         <v>42</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>46</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>45</v>
       </c>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="J4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -892,40 +903,40 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>49</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>100</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>50</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -936,19 +947,19 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>51</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>0.95</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test: add test for OutputPathId resolution producing same result as full path
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\pi-workflow\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F231B5A2-57F5-42D0-9067-256CA473510A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086C4FB0-3C50-4341-B8A9-753F26D5D6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2080" yWindow="960" windowWidth="27640" windowHeight="19270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6960" yWindow="1130" windowWidth="27640" windowHeight="19270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="56">
   <si>
     <t>PITaskName</t>
   </si>
@@ -186,6 +186,12 @@
   </si>
   <si>
     <t>Organism|PeripheralVenousBlood|Aciclovir|Plasma (Peripheral Venous Blood)</t>
+  </si>
+  <si>
+    <t>AciclovirSimplePathId</t>
+  </si>
+  <si>
+    <t>Aciclovir_PVB</t>
   </si>
 </sst>
 </file>
@@ -588,8 +594,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -657,10 +666,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
@@ -692,7 +701,7 @@
         <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>
@@ -724,25 +733,31 @@
         <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>27</v>
+      </c>
+      <c r="E5">
+        <v>-0.1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="H5">
         <v>10</v>
       </c>
       <c r="I5">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -750,7 +765,7 @@
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
         <v>32</v>
@@ -768,6 +783,32 @@
         <v>0.5</v>
       </c>
       <c r="J6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>0.5</v>
+      </c>
+      <c r="J7">
         <v>3</v>
       </c>
     </row>
@@ -779,10 +820,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -843,13 +884,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
         <v>42</v>
@@ -858,7 +899,7 @@
         <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -866,7 +907,7 @@
         <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" t="s">
         <v>53</v>
@@ -875,9 +916,29 @@
         <v>42</v>
       </c>
       <c r="E4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s">
         <v>46</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F5" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: remove unused Value column from PIParameters sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\pi-workflow\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086C4FB0-3C50-4341-B8A9-753F26D5D6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFAB482D-12C3-4C11-AD5A-911D6BDE7DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6960" yWindow="1130" windowWidth="27640" windowHeight="19270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6960" yWindow="1130" windowWidth="27640" windowHeight="19270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="55">
   <si>
     <t>PITaskName</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>Parameter Name</t>
-  </si>
-  <si>
-    <t>Value</t>
   </si>
   <si>
     <t>Units</t>
@@ -594,13 +591,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -628,187 +625,172 @@
       <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="J1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>27</v>
       </c>
-      <c r="E2">
-        <v>-0.1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
+      <c r="F2">
+        <v>-10</v>
       </c>
       <c r="G2">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="H2">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3">
+        <v>-10</v>
+      </c>
+      <c r="G3">
+        <v>10</v>
+      </c>
+      <c r="H3">
         <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3">
-        <v>-0.1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3">
-        <v>-10</v>
-      </c>
-      <c r="H3">
-        <v>10</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
-      <c r="J3">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>-10</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+      <c r="H4">
         <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4">
-        <v>-0.1</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4">
-        <v>-10</v>
-      </c>
-      <c r="H4">
-        <v>10</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
-      <c r="J4">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5">
+        <v>-10</v>
+      </c>
+      <c r="G5">
+        <v>10</v>
+      </c>
+      <c r="H5">
         <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5">
-        <v>-0.1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5">
-        <v>-10</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
         <v>29</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>0.5</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
         <v>32</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6">
+      <c r="F7">
         <v>0</v>
       </c>
-      <c r="H6">
+      <c r="G7">
         <v>10</v>
       </c>
-      <c r="I6">
+      <c r="H7">
         <v>0.5</v>
       </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
       <c r="I7">
-        <v>0.5</v>
-      </c>
-      <c r="J7">
         <v>3</v>
       </c>
     </row>
@@ -835,31 +817,31 @@
         <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>39</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>40</v>
-      </c>
-      <c r="K1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -867,79 +849,79 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" t="s">
         <v>42</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>43</v>
-      </c>
-      <c r="F2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
         <v>54</v>
       </c>
-      <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>55</v>
-      </c>
       <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
         <v>42</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>43</v>
-      </c>
-      <c r="F3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
         <v>42</v>
       </c>
-      <c r="E4" t="s">
-        <v>43</v>
-      </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -958,10 +940,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
         <v>47</v>
-      </c>
-      <c r="C1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -969,7 +951,7 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -980,7 +962,7 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1002,10 +984,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
         <v>47</v>
-      </c>
-      <c r="C1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1013,7 +995,7 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2">
         <v>0.95</v>

</xml_diff>

<commit_message>
chore: reorder PI excel sheets
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/ParameterIdentification.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\pi-workflow\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFAB482D-12C3-4C11-AD5A-911D6BDE7DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642BE751-FE83-4ECD-A435-36791E40D042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6960" yWindow="1130" windowWidth="27640" windowHeight="19270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6960" yWindow="1130" windowWidth="27640" windowHeight="19270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PIConfiguration" sheetId="1" r:id="rId1"/>
+    <sheet name="PIOutputMappings" sheetId="3" r:id="rId1"/>
     <sheet name="PIParameters" sheetId="2" r:id="rId2"/>
-    <sheet name="PIOutputMappings" sheetId="3" r:id="rId3"/>
+    <sheet name="PIConfiguration" sheetId="1" r:id="rId3"/>
     <sheet name="AlgorithmOptions" sheetId="4" r:id="rId4"/>
     <sheet name="CIOptions" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -521,66 +521,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="b">
-        <v>0</v>
+        <v>52</v>
+      </c>
+      <c r="D2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -801,127 +862,66 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.81640625" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" t="s">
-        <v>44</v>
+        <v>15</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>